<commit_message>
refactor: synchronized excel templates and updated backend logic
</commit_message>
<xml_diff>
--- a/app/templates/Template_SALES_SOLUBLES.xlsx
+++ b/app/templates/Template_SALES_SOLUBLES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16479C61-381C-41B7-AAD6-A0775EE94C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4346D05-58EB-40F8-85AF-C09EAC2FE099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,7 +660,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="155">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
@@ -1018,6 +1018,18 @@
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1088,6 +1100,18 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -1112,35 +1136,14 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3774,30 +3777,30 @@
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="128" t="s">
+      <c r="A6" s="132" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="128"/>
-      <c r="C6" s="128"/>
-      <c r="D6" s="128"/>
-      <c r="E6" s="128"/>
-      <c r="F6" s="128"/>
-      <c r="G6" s="128"/>
-      <c r="H6" s="128"/>
-      <c r="I6" s="128"/>
+      <c r="B6" s="132"/>
+      <c r="C6" s="132"/>
+      <c r="D6" s="132"/>
+      <c r="E6" s="132"/>
+      <c r="F6" s="132"/>
+      <c r="G6" s="132"/>
+      <c r="H6" s="132"/>
+      <c r="I6" s="132"/>
     </row>
     <row r="7" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="129" t="s">
+      <c r="A7" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="129"/>
-      <c r="C7" s="129"/>
-      <c r="D7" s="129"/>
-      <c r="E7" s="129"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="129"/>
-      <c r="I7" s="129"/>
+      <c r="B7" s="133"/>
+      <c r="C7" s="133"/>
+      <c r="D7" s="133"/>
+      <c r="E7" s="133"/>
+      <c r="F7" s="133"/>
+      <c r="G7" s="133"/>
+      <c r="H7" s="133"/>
+      <c r="I7" s="133"/>
     </row>
     <row r="8" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="29"/>
@@ -3849,32 +3852,32 @@
       <c r="K11" s="15"/>
     </row>
     <row r="12" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="130" t="s">
+      <c r="A12" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="131"/>
-      <c r="C12" s="131"/>
-      <c r="D12" s="131"/>
-      <c r="E12" s="131"/>
-      <c r="F12" s="131"/>
-      <c r="G12" s="131"/>
-      <c r="H12" s="131"/>
-      <c r="I12" s="132"/>
+      <c r="B12" s="135"/>
+      <c r="C12" s="135"/>
+      <c r="D12" s="135"/>
+      <c r="E12" s="135"/>
+      <c r="F12" s="135"/>
+      <c r="G12" s="135"/>
+      <c r="H12" s="135"/>
+      <c r="I12" s="136"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
     </row>
     <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="125" t="s">
+      <c r="A13" s="129" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="126"/>
-      <c r="C13" s="126"/>
-      <c r="D13" s="126"/>
-      <c r="E13" s="126"/>
-      <c r="F13" s="126"/>
-      <c r="G13" s="126"/>
-      <c r="H13" s="126"/>
-      <c r="I13" s="127"/>
+      <c r="B13" s="130"/>
+      <c r="C13" s="130"/>
+      <c r="D13" s="130"/>
+      <c r="E13" s="130"/>
+      <c r="F13" s="130"/>
+      <c r="G13" s="130"/>
+      <c r="H13" s="130"/>
+      <c r="I13" s="131"/>
       <c r="J13" s="15"/>
       <c r="K13" s="15"/>
     </row>
@@ -3892,11 +3895,11 @@
       <c r="K14" s="15"/>
     </row>
     <row r="15" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="134"/>
-      <c r="D15" s="134"/>
-      <c r="E15" s="134"/>
-      <c r="G15" s="134"/>
-      <c r="H15" s="134"/>
+      <c r="C15" s="138"/>
+      <c r="D15" s="138"/>
+      <c r="E15" s="138"/>
+      <c r="G15" s="138"/>
+      <c r="H15" s="138"/>
       <c r="I15" s="53"/>
       <c r="K15" s="15"/>
     </row>
@@ -3930,17 +3933,17 @@
       <c r="K18" s="15"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="135" t="s">
+      <c r="A19" s="139" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="136"/>
-      <c r="C19" s="136"/>
-      <c r="D19" s="136"/>
-      <c r="E19" s="136"/>
-      <c r="F19" s="136"/>
-      <c r="G19" s="136"/>
-      <c r="H19" s="136"/>
-      <c r="I19" s="137"/>
+      <c r="B19" s="140"/>
+      <c r="C19" s="140"/>
+      <c r="D19" s="140"/>
+      <c r="E19" s="140"/>
+      <c r="F19" s="140"/>
+      <c r="G19" s="140"/>
+      <c r="H19" s="140"/>
+      <c r="I19" s="141"/>
       <c r="K19" s="15"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4119,17 +4122,17 @@
       <c r="K29" s="15"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="135" t="s">
+      <c r="A30" s="139" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="136"/>
-      <c r="C30" s="136"/>
-      <c r="D30" s="136"/>
-      <c r="E30" s="136"/>
-      <c r="F30" s="136"/>
-      <c r="G30" s="136"/>
-      <c r="H30" s="136"/>
-      <c r="I30" s="137"/>
+      <c r="B30" s="140"/>
+      <c r="C30" s="140"/>
+      <c r="D30" s="140"/>
+      <c r="E30" s="140"/>
+      <c r="F30" s="140"/>
+      <c r="G30" s="140"/>
+      <c r="H30" s="140"/>
+      <c r="I30" s="141"/>
       <c r="J30" s="15"/>
       <c r="K30" s="15"/>
     </row>
@@ -4245,14 +4248,14 @@
     <row r="38" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="91"/>
       <c r="B38" s="44"/>
-      <c r="C38" s="118" t="s">
+      <c r="C38" s="122" t="s">
         <v>46</v>
       </c>
-      <c r="D38" s="119"/>
-      <c r="E38" s="119"/>
-      <c r="F38" s="119"/>
-      <c r="G38" s="119"/>
-      <c r="H38" s="120"/>
+      <c r="D38" s="123"/>
+      <c r="E38" s="123"/>
+      <c r="F38" s="123"/>
+      <c r="G38" s="123"/>
+      <c r="H38" s="124"/>
       <c r="I38" s="36"/>
       <c r="J38" s="15"/>
       <c r="K38" s="15"/>
@@ -4260,12 +4263,12 @@
     <row r="39" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="91"/>
       <c r="B39" s="44"/>
-      <c r="C39" s="121"/>
-      <c r="D39" s="122"/>
-      <c r="E39" s="122"/>
-      <c r="F39" s="122"/>
-      <c r="G39" s="122"/>
-      <c r="H39" s="123"/>
+      <c r="C39" s="125"/>
+      <c r="D39" s="126"/>
+      <c r="E39" s="126"/>
+      <c r="F39" s="126"/>
+      <c r="G39" s="126"/>
+      <c r="H39" s="127"/>
       <c r="I39" s="36"/>
       <c r="J39" s="15"/>
       <c r="K39" s="15"/>
@@ -4425,12 +4428,12 @@
       <c r="K51" s="15"/>
     </row>
     <row r="52" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="133"/>
-      <c r="C52" s="133"/>
-      <c r="D52" s="133"/>
-      <c r="E52" s="133"/>
-      <c r="F52" s="133"/>
-      <c r="G52" s="133"/>
+      <c r="B52" s="137"/>
+      <c r="C52" s="137"/>
+      <c r="D52" s="137"/>
+      <c r="E52" s="137"/>
+      <c r="F52" s="137"/>
+      <c r="G52" s="137"/>
       <c r="H52" s="38"/>
       <c r="I52" s="14"/>
       <c r="J52" s="15"/>
@@ -4468,17 +4471,17 @@
     </row>
     <row r="55" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="124" t="s">
+      <c r="A56" s="128" t="s">
         <v>17</v>
       </c>
-      <c r="B56" s="124"/>
-      <c r="C56" s="124"/>
-      <c r="D56" s="124"/>
-      <c r="E56" s="124"/>
-      <c r="F56" s="124"/>
-      <c r="G56" s="124"/>
-      <c r="H56" s="124"/>
-      <c r="I56" s="124"/>
+      <c r="B56" s="128"/>
+      <c r="C56" s="128"/>
+      <c r="D56" s="128"/>
+      <c r="E56" s="128"/>
+      <c r="F56" s="128"/>
+      <c r="G56" s="128"/>
+      <c r="H56" s="128"/>
+      <c r="I56" s="128"/>
     </row>
     <row r="57" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4583,30 +4586,30 @@
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="128" t="s">
+      <c r="A6" s="132" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="128"/>
-      <c r="C6" s="128"/>
-      <c r="D6" s="128"/>
-      <c r="E6" s="128"/>
-      <c r="F6" s="128"/>
-      <c r="G6" s="128"/>
-      <c r="H6" s="128"/>
-      <c r="I6" s="128"/>
+      <c r="B6" s="132"/>
+      <c r="C6" s="132"/>
+      <c r="D6" s="132"/>
+      <c r="E6" s="132"/>
+      <c r="F6" s="132"/>
+      <c r="G6" s="132"/>
+      <c r="H6" s="132"/>
+      <c r="I6" s="132"/>
     </row>
     <row r="7" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="129" t="s">
+      <c r="A7" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="129"/>
-      <c r="C7" s="129"/>
-      <c r="D7" s="129"/>
-      <c r="E7" s="129"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="129"/>
-      <c r="I7" s="129"/>
+      <c r="B7" s="133"/>
+      <c r="C7" s="133"/>
+      <c r="D7" s="133"/>
+      <c r="E7" s="133"/>
+      <c r="F7" s="133"/>
+      <c r="G7" s="133"/>
+      <c r="H7" s="133"/>
+      <c r="I7" s="133"/>
     </row>
     <row r="8" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="29"/>
@@ -4615,34 +4618,34 @@
       <c r="M8"/>
     </row>
     <row r="9" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="145" t="s">
+      <c r="B9" s="152" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="145"/>
-      <c r="D9" s="146" t="s">
+      <c r="C9" s="152"/>
+      <c r="D9" s="118" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="148" t="s">
+      <c r="E9" s="144" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="149"/>
-      <c r="G9" s="148" t="s">
+      <c r="F9" s="145"/>
+      <c r="G9" s="144" t="s">
         <v>60</v>
       </c>
-      <c r="H9" s="149"/>
+      <c r="H9" s="145"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9" s="15"/>
     </row>
     <row r="10" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="37"/>
-      <c r="B10" s="150"/>
-      <c r="C10" s="151"/>
-      <c r="D10" s="147"/>
-      <c r="E10" s="152"/>
-      <c r="F10" s="153"/>
-      <c r="G10" s="152"/>
-      <c r="H10" s="153"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="143"/>
+      <c r="D10" s="119"/>
+      <c r="E10" s="120"/>
+      <c r="F10" s="121"/>
+      <c r="G10" s="120"/>
+      <c r="H10" s="121"/>
       <c r="I10" s="39"/>
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
@@ -4661,32 +4664,32 @@
       <c r="K11" s="15"/>
     </row>
     <row r="12" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="130" t="s">
+      <c r="A12" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="131"/>
-      <c r="C12" s="131"/>
-      <c r="D12" s="131"/>
-      <c r="E12" s="131"/>
-      <c r="F12" s="131"/>
-      <c r="G12" s="131"/>
-      <c r="H12" s="131"/>
-      <c r="I12" s="132"/>
+      <c r="B12" s="135"/>
+      <c r="C12" s="135"/>
+      <c r="D12" s="135"/>
+      <c r="E12" s="135"/>
+      <c r="F12" s="135"/>
+      <c r="G12" s="135"/>
+      <c r="H12" s="135"/>
+      <c r="I12" s="136"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
     </row>
     <row r="13" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="125" t="s">
+      <c r="A13" s="129" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="126"/>
-      <c r="C13" s="126"/>
-      <c r="D13" s="126"/>
-      <c r="E13" s="126"/>
-      <c r="F13" s="126"/>
-      <c r="G13" s="126"/>
-      <c r="H13" s="126"/>
-      <c r="I13" s="127"/>
+      <c r="B13" s="130"/>
+      <c r="C13" s="130"/>
+      <c r="D13" s="130"/>
+      <c r="E13" s="130"/>
+      <c r="F13" s="130"/>
+      <c r="G13" s="130"/>
+      <c r="H13" s="130"/>
+      <c r="I13" s="131"/>
       <c r="J13" s="15"/>
       <c r="K13" s="15"/>
     </row>
@@ -4704,11 +4707,11 @@
       <c r="K14" s="15"/>
     </row>
     <row r="15" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="134"/>
-      <c r="D15" s="134"/>
-      <c r="E15" s="134"/>
-      <c r="G15" s="134"/>
-      <c r="H15" s="134"/>
+      <c r="C15" s="138"/>
+      <c r="D15" s="138"/>
+      <c r="E15" s="138"/>
+      <c r="G15" s="138"/>
+      <c r="H15" s="138"/>
       <c r="I15" s="53"/>
       <c r="K15" s="15"/>
     </row>
@@ -4742,17 +4745,17 @@
       <c r="K18" s="15"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="135" t="s">
+      <c r="A19" s="139" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="136"/>
-      <c r="C19" s="136"/>
-      <c r="D19" s="136"/>
-      <c r="E19" s="136"/>
-      <c r="F19" s="136"/>
-      <c r="G19" s="136"/>
-      <c r="H19" s="136"/>
-      <c r="I19" s="137"/>
+      <c r="B19" s="140"/>
+      <c r="C19" s="140"/>
+      <c r="D19" s="140"/>
+      <c r="E19" s="140"/>
+      <c r="F19" s="140"/>
+      <c r="G19" s="140"/>
+      <c r="H19" s="140"/>
+      <c r="I19" s="141"/>
       <c r="K19" s="15"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4778,8 +4781,8 @@
       <c r="F21" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="G21" s="81"/>
-      <c r="H21" s="81"/>
+      <c r="G21" s="154"/>
+      <c r="H21" s="154"/>
       <c r="I21" s="80"/>
       <c r="J21" s="15"/>
       <c r="K21" s="31"/>
@@ -4931,17 +4934,17 @@
       <c r="K29" s="15"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="135" t="s">
+      <c r="A30" s="139" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="136"/>
-      <c r="C30" s="136"/>
-      <c r="D30" s="136"/>
-      <c r="E30" s="136"/>
-      <c r="F30" s="136"/>
-      <c r="G30" s="136"/>
-      <c r="H30" s="136"/>
-      <c r="I30" s="137"/>
+      <c r="B30" s="140"/>
+      <c r="C30" s="140"/>
+      <c r="D30" s="140"/>
+      <c r="E30" s="140"/>
+      <c r="F30" s="140"/>
+      <c r="G30" s="140"/>
+      <c r="H30" s="140"/>
+      <c r="I30" s="141"/>
       <c r="J30" s="15"/>
       <c r="K30" s="15"/>
     </row>
@@ -5057,14 +5060,14 @@
     <row r="38" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="91"/>
       <c r="B38" s="44"/>
-      <c r="C38" s="118" t="s">
+      <c r="C38" s="122" t="s">
         <v>46</v>
       </c>
-      <c r="D38" s="119"/>
-      <c r="E38" s="119"/>
-      <c r="F38" s="119"/>
-      <c r="G38" s="119"/>
-      <c r="H38" s="120"/>
+      <c r="D38" s="123"/>
+      <c r="E38" s="123"/>
+      <c r="F38" s="123"/>
+      <c r="G38" s="123"/>
+      <c r="H38" s="124"/>
       <c r="I38" s="36"/>
       <c r="J38" s="15"/>
       <c r="K38" s="15"/>
@@ -5072,12 +5075,12 @@
     <row r="39" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="91"/>
       <c r="B39" s="44"/>
-      <c r="C39" s="121"/>
-      <c r="D39" s="122"/>
-      <c r="E39" s="122"/>
-      <c r="F39" s="122"/>
-      <c r="G39" s="122"/>
-      <c r="H39" s="123"/>
+      <c r="C39" s="125"/>
+      <c r="D39" s="126"/>
+      <c r="E39" s="126"/>
+      <c r="F39" s="126"/>
+      <c r="G39" s="126"/>
+      <c r="H39" s="127"/>
       <c r="I39" s="36"/>
       <c r="J39" s="15"/>
       <c r="K39" s="15"/>
@@ -5111,14 +5114,14 @@
     <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="43"/>
       <c r="B42" s="43"/>
-      <c r="C42" s="142" t="s">
+      <c r="C42" s="150" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="143"/>
-      <c r="E42" s="142" t="s">
+      <c r="D42" s="151"/>
+      <c r="E42" s="150" t="s">
         <v>51</v>
       </c>
-      <c r="F42" s="143"/>
+      <c r="F42" s="151"/>
       <c r="G42" s="110"/>
       <c r="H42" s="110"/>
       <c r="I42" s="43"/>
@@ -5128,12 +5131,12 @@
     <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="43"/>
       <c r="B43" s="43"/>
-      <c r="C43" s="138" t="s">
+      <c r="C43" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="139"/>
-      <c r="E43" s="140"/>
-      <c r="F43" s="141"/>
+      <c r="D43" s="147"/>
+      <c r="E43" s="148"/>
+      <c r="F43" s="149"/>
       <c r="G43" s="110"/>
       <c r="H43" s="110"/>
       <c r="I43" s="43"/>
@@ -5143,12 +5146,12 @@
     <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="43"/>
       <c r="B44" s="43"/>
-      <c r="C44" s="138" t="s">
+      <c r="C44" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="D44" s="139"/>
-      <c r="E44" s="140"/>
-      <c r="F44" s="141"/>
+      <c r="D44" s="147"/>
+      <c r="E44" s="148"/>
+      <c r="F44" s="149"/>
       <c r="G44" s="110"/>
       <c r="H44" s="110"/>
       <c r="I44" s="43"/>
@@ -5158,12 +5161,12 @@
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="43"/>
       <c r="B45" s="43"/>
-      <c r="C45" s="138" t="s">
+      <c r="C45" s="146" t="s">
         <v>56</v>
       </c>
-      <c r="D45" s="139"/>
-      <c r="E45" s="140"/>
-      <c r="F45" s="141"/>
+      <c r="D45" s="147"/>
+      <c r="E45" s="148"/>
+      <c r="F45" s="149"/>
       <c r="G45" s="110"/>
       <c r="H45" s="110"/>
       <c r="I45" s="43"/>
@@ -5243,12 +5246,12 @@
       <c r="K51" s="15"/>
     </row>
     <row r="52" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="133"/>
-      <c r="C52" s="133"/>
-      <c r="D52" s="133"/>
-      <c r="E52" s="133"/>
-      <c r="F52" s="133"/>
-      <c r="G52" s="133"/>
+      <c r="B52" s="137"/>
+      <c r="C52" s="137"/>
+      <c r="D52" s="137"/>
+      <c r="E52" s="137"/>
+      <c r="F52" s="137"/>
+      <c r="G52" s="137"/>
       <c r="H52" s="38"/>
       <c r="I52" s="14"/>
       <c r="J52" s="15"/>
@@ -5287,17 +5290,17 @@
     </row>
     <row r="55" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="124" t="s">
+      <c r="A56" s="128" t="s">
         <v>17</v>
       </c>
-      <c r="B56" s="124"/>
-      <c r="C56" s="124"/>
-      <c r="D56" s="124"/>
-      <c r="E56" s="124"/>
-      <c r="F56" s="124"/>
-      <c r="G56" s="124"/>
-      <c r="H56" s="124"/>
-      <c r="I56" s="124"/>
+      <c r="B56" s="128"/>
+      <c r="C56" s="128"/>
+      <c r="D56" s="128"/>
+      <c r="E56" s="128"/>
+      <c r="F56" s="128"/>
+      <c r="G56" s="128"/>
+      <c r="H56" s="128"/>
+      <c r="I56" s="128"/>
     </row>
     <row r="57" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5307,11 +5310,14 @@
     <protectedRange sqref="C52" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="24">
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="B9:C9"/>
     <mergeCell ref="C38:H39"/>
     <mergeCell ref="B52:D52"/>
     <mergeCell ref="E52:G52"/>
@@ -5319,18 +5325,15 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B9:C9"/>
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="E44:F44"/>
-    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A30:I30"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -5357,10 +5360,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="144" t="s">
+      <c r="A2" s="153" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="144"/>
+      <c r="B2" s="153"/>
       <c r="C2" s="6" t="s">
         <v>10</v>
       </c>

</xml_diff>